<commit_message>
Add points for 66cem7lh6o8ckkfxp4tao7o5w_playerlog
</commit_message>
<xml_diff>
--- a/bnc-streamlit-app/data/points/66cem7lh6o8ckkfxp4tao7o5w_playerlog.xlsx
+++ b/bnc-streamlit-app/data/points/66cem7lh6o8ckkfxp4tao7o5w_playerlog.xlsx
@@ -1008,11 +1008,11 @@
         </is>
       </c>
       <c r="AI3" t="n">
-        <v>2.01945437</v>
+        <v>2.0379362</v>
       </c>
       <c r="AJ3" t="inlineStr">
         <is>
-          <t>+1.22</t>
+          <t>+1.23</t>
         </is>
       </c>
       <c r="AK3" t="n">
@@ -1195,15 +1195,15 @@
         </is>
       </c>
       <c r="AI4" t="n">
-        <v>1.98261648</v>
+        <v>1.9851343</v>
       </c>
       <c r="AJ4" t="inlineStr">
         <is>
-          <t>+1.19</t>
+          <t>+1.18</t>
         </is>
       </c>
       <c r="AK4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AL4" t="n">
         <v>0</v>
@@ -1384,11 +1384,11 @@
         </is>
       </c>
       <c r="AI5" t="n">
-        <v>2.30381861</v>
+        <v>2.34456471</v>
       </c>
       <c r="AJ5" t="inlineStr">
         <is>
-          <t>+1.51</t>
+          <t>+1.54</t>
         </is>
       </c>
       <c r="AK5" t="n">
@@ -1422,7 +1422,7 @@
         <v>0</v>
       </c>
       <c r="AU5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AV5" t="n">
         <v>0</v>
@@ -1454,7 +1454,7 @@
         </is>
       </c>
       <c r="BE5" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="BF5" t="n">
         <v>3</v>
@@ -1571,11 +1571,11 @@
         </is>
       </c>
       <c r="AI6" t="n">
-        <v>1.59154314</v>
+        <v>1.59205356</v>
       </c>
       <c r="AJ6" t="inlineStr">
         <is>
-          <t>+0.79</t>
+          <t>+0.78</t>
         </is>
       </c>
       <c r="AK6" t="n">
@@ -1758,15 +1758,15 @@
         </is>
       </c>
       <c r="AI7" t="n">
-        <v>1.85107267</v>
+        <v>2.09225782</v>
       </c>
       <c r="AJ7" t="inlineStr">
         <is>
-          <t>+1.05</t>
+          <t>+1.28</t>
         </is>
       </c>
       <c r="AK7" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="AL7" t="n">
         <v>0</v>
@@ -1947,11 +1947,11 @@
         </is>
       </c>
       <c r="AI8" t="n">
-        <v>1.43583423</v>
+        <v>1.39535187</v>
       </c>
       <c r="AJ8" t="inlineStr">
         <is>
-          <t>+0.64</t>
+          <t>+0.59</t>
         </is>
       </c>
       <c r="AK8" t="n">
@@ -1985,7 +1985,7 @@
         <v>1</v>
       </c>
       <c r="AU8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AV8" t="n">
         <v>0</v>
@@ -2017,7 +2017,7 @@
         </is>
       </c>
       <c r="BE8" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="BF8" t="n">
         <v>1</v>
@@ -2144,11 +2144,11 @@
         </is>
       </c>
       <c r="AI9" t="n">
-        <v>2.40897677</v>
+        <v>2.39487215</v>
       </c>
       <c r="AJ9" t="inlineStr">
         <is>
-          <t>+1.61</t>
+          <t>+1.59</t>
         </is>
       </c>
       <c r="AK9" t="n">
@@ -2335,7 +2335,7 @@
       </c>
       <c r="AJ10" t="inlineStr">
         <is>
-          <t>+0.34</t>
+          <t>+0.33</t>
         </is>
       </c>
       <c r="AK10" t="n">
@@ -2357,7 +2357,7 @@
         <v>1</v>
       </c>
       <c r="AQ10" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AR10" t="n">
         <v>0</v>
@@ -2404,7 +2404,7 @@
         <v>1</v>
       </c>
       <c r="BF10" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="BG10" t="n">
         <v>2</v>
@@ -2530,15 +2530,15 @@
         </is>
       </c>
       <c r="AI11" t="n">
-        <v>1.30777651</v>
+        <v>1.3801799</v>
       </c>
       <c r="AJ11" t="inlineStr">
         <is>
-          <t>+0.51</t>
+          <t>+0.57</t>
         </is>
       </c>
       <c r="AK11" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="AL11" t="n">
         <v>0</v>
@@ -2553,13 +2553,13 @@
         <v>0</v>
       </c>
       <c r="AP11" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AQ11" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AR11" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="AS11" t="n">
         <v>0</v>
@@ -2600,7 +2600,7 @@
         </is>
       </c>
       <c r="BE11" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="BF11" t="n">
         <v>4</v>
@@ -2719,11 +2719,11 @@
         </is>
       </c>
       <c r="AI12" t="n">
-        <v>0.48463769</v>
+        <v>0.48212117</v>
       </c>
       <c r="AJ12" t="inlineStr">
         <is>
-          <t>-0.31</t>
+          <t>-0.33</t>
         </is>
       </c>
       <c r="AK12" t="n">
@@ -2920,7 +2920,7 @@
       </c>
       <c r="AJ13" t="inlineStr">
         <is>
-          <t>-0.13</t>
+          <t>-0.14</t>
         </is>
       </c>
       <c r="AK13" t="n">
@@ -3117,7 +3117,7 @@
       </c>
       <c r="AJ14" t="inlineStr">
         <is>
-          <t>-0.53</t>
+          <t>-0.54</t>
         </is>
       </c>
       <c r="AK14" t="n">
@@ -3318,7 +3318,7 @@
       </c>
       <c r="AJ15" t="inlineStr">
         <is>
-          <t>-0.78</t>
+          <t>-0.79</t>
         </is>
       </c>
       <c r="AK15" t="n">
@@ -3505,11 +3505,11 @@
         </is>
       </c>
       <c r="AI16" t="n">
-        <v>0.69829235</v>
+        <v>0.6973116499999999</v>
       </c>
       <c r="AJ16" t="inlineStr">
         <is>
-          <t>-0.10</t>
+          <t>-0.11</t>
         </is>
       </c>
       <c r="AK16" t="n">
@@ -3867,7 +3867,7 @@
       </c>
       <c r="AJ18" t="inlineStr">
         <is>
-          <t>-0.24</t>
+          <t>-0.25</t>
         </is>
       </c>
       <c r="AK18" t="n">
@@ -4048,11 +4048,11 @@
         </is>
       </c>
       <c r="AI19" t="n">
-        <v>0.19450252</v>
+        <v>0.03153339000000002</v>
       </c>
       <c r="AJ19" t="inlineStr">
         <is>
-          <t>-0.60</t>
+          <t>-0.78</t>
         </is>
       </c>
       <c r="AK19" t="n">
@@ -4074,16 +4074,16 @@
         <v>1</v>
       </c>
       <c r="AQ19" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AR19" t="n">
         <v>5</v>
       </c>
       <c r="AS19" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="AT19" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="AU19" t="n">
         <v>2</v>
@@ -4117,7 +4117,7 @@
         <v>0</v>
       </c>
       <c r="BF19" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="BG19" t="n">
         <v>0</v>
@@ -4231,11 +4231,11 @@
         </is>
       </c>
       <c r="AI20" t="n">
-        <v>0.26037628</v>
+        <v>0.2609581400000001</v>
       </c>
       <c r="AJ20" t="inlineStr">
         <is>
-          <t>-0.54</t>
+          <t>-0.55</t>
         </is>
       </c>
       <c r="AK20" t="n">
@@ -4414,15 +4414,15 @@
         </is>
       </c>
       <c r="AI21" t="n">
-        <v>2.03027363</v>
+        <v>2.0303297</v>
       </c>
       <c r="AJ21" t="inlineStr">
         <is>
-          <t>+1.23</t>
+          <t>+1.22</t>
         </is>
       </c>
       <c r="AK21" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="AL21" t="n">
         <v>0</v>
@@ -4597,15 +4597,15 @@
         </is>
       </c>
       <c r="AI22" t="n">
-        <v>1.3158405</v>
+        <v>1.35969865</v>
       </c>
       <c r="AJ22" t="inlineStr">
         <is>
-          <t>+0.52</t>
+          <t>+0.55</t>
         </is>
       </c>
       <c r="AK22" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="AL22" t="n">
         <v>0</v>
@@ -4780,11 +4780,11 @@
         </is>
       </c>
       <c r="AI23" t="n">
-        <v>0.69517442</v>
+        <v>0.6948202300000001</v>
       </c>
       <c r="AJ23" t="inlineStr">
         <is>
-          <t>-0.10</t>
+          <t>-0.11</t>
         </is>
       </c>
       <c r="AK23" t="n">
@@ -4969,7 +4969,7 @@
       </c>
       <c r="AJ24" t="inlineStr">
         <is>
-          <t>-0.89</t>
+          <t>-0.90</t>
         </is>
       </c>
       <c r="AK24" t="n">
@@ -5154,7 +5154,7 @@
       </c>
       <c r="AJ25" t="inlineStr">
         <is>
-          <t>-0.78</t>
+          <t>-0.79</t>
         </is>
       </c>
       <c r="AK25" t="n">
@@ -5335,7 +5335,7 @@
         </is>
       </c>
       <c r="AI26" t="n">
-        <v>-0.24155551</v>
+        <v>-0.23085297</v>
       </c>
       <c r="AJ26" t="inlineStr">
         <is>
@@ -5343,7 +5343,7 @@
         </is>
       </c>
       <c r="AK26" t="n">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="AL26" t="n">
         <v>0</v>
@@ -5364,7 +5364,7 @@
         <v>2</v>
       </c>
       <c r="AR26" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="AS26" t="n">
         <v>2</v>
@@ -5520,15 +5520,15 @@
         </is>
       </c>
       <c r="AI27" t="n">
-        <v>0.32094362</v>
+        <v>0.40165715</v>
       </c>
       <c r="AJ27" t="inlineStr">
         <is>
-          <t>-0.48</t>
+          <t>-0.41</t>
         </is>
       </c>
       <c r="AK27" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="AL27" t="n">
         <v>0</v>
@@ -5558,7 +5558,7 @@
         <v>1</v>
       </c>
       <c r="AU27" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AV27" t="n">
         <v>0</v>
@@ -5711,7 +5711,7 @@
       </c>
       <c r="AJ28" t="inlineStr">
         <is>
-          <t>-0.56</t>
+          <t>-0.57</t>
         </is>
       </c>
       <c r="AK28" t="n">
@@ -5898,11 +5898,11 @@
       </c>
       <c r="AJ29" t="inlineStr">
         <is>
-          <t>-0.40</t>
+          <t>-0.42</t>
         </is>
       </c>
       <c r="AK29" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="AL29" t="n">
         <v>60</v>
@@ -6081,15 +6081,15 @@
         </is>
       </c>
       <c r="AI30" t="n">
-        <v>-0.22277608</v>
+        <v>-0.23440257</v>
       </c>
       <c r="AJ30" t="inlineStr">
         <is>
-          <t>-1.02</t>
+          <t>-1.04</t>
         </is>
       </c>
       <c r="AK30" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="AL30" t="n">
         <v>60</v>
@@ -6272,7 +6272,7 @@
       </c>
       <c r="AJ31" t="inlineStr">
         <is>
-          <t>-0.59</t>
+          <t>-0.60</t>
         </is>
       </c>
       <c r="AK31" t="n">
@@ -6459,7 +6459,7 @@
       </c>
       <c r="AJ32" t="inlineStr">
         <is>
-          <t>-0.94</t>
+          <t>-0.95</t>
         </is>
       </c>
       <c r="AK32" t="n">

</xml_diff>